<commit_message>
Drop phase subtotals and the deliverable column from the CAN plan.
Co-authored-by: feartreefeartree-ux <feartreefeartree-ux@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/CAN/FAN_F-SW-100_高压风扇CAN开发计划.xlsx
+++ b/docs/CAN/FAN_F-SW-100_高压风扇CAN开发计划.xlsx
@@ -10,7 +10,7 @@
     <sheet name="工作任务分解" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'工作任务分解'!$A$4:$H$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'工作任务分解'!$A$4:$G$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'工作任务分解'!$1:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -57,7 +57,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -97,17 +97,6 @@
         <color rgb="00808080"/>
       </top>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00808080"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00808080"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -160,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -178,15 +167,11 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -552,17 +537,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H55"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="33" customHeight="1">
@@ -577,7 +561,6 @@
       <c r="E1" s="2" t="n"/>
       <c r="F1" s="2" t="n"/>
       <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -606,12 +589,7 @@
           <t>V1.2</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>日期</t>
-        </is>
-      </c>
-      <c r="H2" s="5" t="n">
+      <c r="G2" s="5" t="n">
         <v>46279</v>
       </c>
     </row>
@@ -635,7 +613,6 @@
       </c>
       <c r="F3" s="4" t="inlineStr"/>
       <c r="G3" s="6" t="n"/>
-      <c r="H3" s="7" t="n"/>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -673,11 +650,6 @@
           <t>负责人</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>交付物</t>
-        </is>
-      </c>
     </row>
     <row r="5" ht="33" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -690,7 +662,7 @@
           <t>需求分析与评审</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>客户资料分析与需求拆解</t>
         </is>
@@ -707,11 +679,6 @@
           <t>系统工程师</t>
         </is>
       </c>
-      <c r="H5" s="8" t="inlineStr">
-        <is>
-          <t>D01 系统需求规格书</t>
-        </is>
-      </c>
     </row>
     <row r="6" ht="33" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
@@ -719,8 +686,8 @@
           <t>1.2</t>
         </is>
       </c>
-      <c r="B6" s="9" t="n"/>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="B6" s="8" t="n"/>
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>需求拆解表编制</t>
         </is>
@@ -737,11 +704,6 @@
           <t>系统工程师</t>
         </is>
       </c>
-      <c r="H6" s="8" t="inlineStr">
-        <is>
-          <t>D02 需求拆解表</t>
-        </is>
-      </c>
     </row>
     <row r="7" ht="33" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -749,8 +711,8 @@
           <t>1.3</t>
         </is>
       </c>
-      <c r="B7" s="9" t="n"/>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="B7" s="8" t="n"/>
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>需求评审会议</t>
         </is>
@@ -767,11 +729,6 @@
           <t>项目经理+系统工程师</t>
         </is>
       </c>
-      <c r="H7" s="8" t="inlineStr">
-        <is>
-          <t>D03 需求评审记录表</t>
-        </is>
-      </c>
     </row>
     <row r="8" ht="33" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
@@ -779,8 +736,8 @@
           <t>1.4</t>
         </is>
       </c>
-      <c r="B8" s="9" t="n"/>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="B8" s="8" t="n"/>
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>芯片可行性确认</t>
         </is>
@@ -797,11 +754,6 @@
           <t>系统工程师</t>
         </is>
       </c>
-      <c r="H8" s="8" t="inlineStr">
-        <is>
-          <t>芯片可行性分析报告</t>
-        </is>
-      </c>
     </row>
     <row r="9" ht="33" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
@@ -809,8 +761,8 @@
           <t>1.5</t>
         </is>
       </c>
-      <c r="B9" s="10" t="n"/>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="B9" s="9" t="n"/>
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>CAN 矩阵 / DBC 冻结</t>
         </is>
@@ -831,81 +783,78 @@
           <t>系统工程师</t>
         </is>
       </c>
-      <c r="H9" s="8" t="inlineStr">
-        <is>
-          <t>已确认矩阵 / DBC 版本</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="16.5" customHeight="1">
-      <c r="A10" s="3" t="inlineStr"/>
-      <c r="B10" s="3" t="inlineStr"/>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>阶段一 小计</t>
-        </is>
-      </c>
-      <c r="D10" s="11" t="n">
-        <v>46188</v>
-      </c>
-      <c r="E10" s="11" t="n">
-        <v>46199</v>
+    </row>
+    <row r="10" ht="33" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>架构与详细设计</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>软件架构设计</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>46202</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>46203</v>
       </c>
       <c r="F10" s="4" t="inlineStr"/>
-      <c r="G10" s="4" t="inlineStr"/>
-      <c r="H10" s="4" t="inlineStr"/>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>系统工程师</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="33" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>2.1</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>架构与详细设计</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>软件架构设计</t>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="n"/>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Bootloader 详细设计</t>
         </is>
       </c>
       <c r="D11" s="5" t="n">
-        <v>46202</v>
+        <v>46204</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>46203</v>
+        <v>46205</v>
       </c>
       <c r="F11" s="4" t="inlineStr"/>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>系统工程师</t>
-        </is>
-      </c>
-      <c r="H11" s="8" t="inlineStr">
-        <is>
-          <t>D04 软件架构设计文档</t>
+          <t>嵌入式开发工程师</t>
         </is>
       </c>
     </row>
     <row r="12" ht="33" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>2.2</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="n"/>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>Bootloader 详细设计</t>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="n"/>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>UDS 诊断栈详细设计</t>
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>46204</v>
+        <v>46206</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>46205</v>
+        <v>46209</v>
       </c>
       <c r="F12" s="4" t="inlineStr"/>
       <c r="G12" s="4" t="inlineStr">
@@ -913,29 +862,24 @@
           <t>嵌入式开发工程师</t>
         </is>
       </c>
-      <c r="H12" s="8" t="inlineStr">
-        <is>
-          <t>D05 Bootloader 详细设计</t>
-        </is>
-      </c>
     </row>
     <row r="13" ht="33" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>2.3</t>
-        </is>
-      </c>
-      <c r="B13" s="9" t="n"/>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>UDS 诊断栈详细设计</t>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="n"/>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>安全访问模块设计</t>
         </is>
       </c>
       <c r="D13" s="5" t="n">
-        <v>46206</v>
+        <v>46210</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>46209</v>
+        <v>46211</v>
       </c>
       <c r="F13" s="4" t="inlineStr"/>
       <c r="G13" s="4" t="inlineStr">
@@ -943,29 +887,24 @@
           <t>嵌入式开发工程师</t>
         </is>
       </c>
-      <c r="H13" s="8" t="inlineStr">
-        <is>
-          <t>D06 UDS 诊断栈详细设计</t>
-        </is>
-      </c>
     </row>
     <row r="14" ht="33" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>2.4</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="n"/>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>安全访问模块设计</t>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="n"/>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Flash 分区与存储管理设计</t>
         </is>
       </c>
       <c r="D14" s="5" t="n">
-        <v>46210</v>
+        <v>46212</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
       <c r="F14" s="4" t="inlineStr"/>
       <c r="G14" s="4" t="inlineStr">
@@ -973,29 +912,24 @@
           <t>嵌入式开发工程师</t>
         </is>
       </c>
-      <c r="H14" s="8" t="inlineStr">
-        <is>
-          <t>D07 安全访问设计</t>
-        </is>
-      </c>
     </row>
     <row r="15" ht="33" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>2.5</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="n"/>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>Flash 分区与存储管理设计</t>
+          <t>2.6</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="n"/>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>CAN 通信设计</t>
         </is>
       </c>
       <c r="D15" s="5" t="n">
-        <v>46212</v>
+        <v>46216</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>46213</v>
+        <v>46217</v>
       </c>
       <c r="F15" s="4" t="inlineStr"/>
       <c r="G15" s="4" t="inlineStr">
@@ -1003,111 +937,103 @@
           <t>嵌入式开发工程师</t>
         </is>
       </c>
-      <c r="H15" s="8" t="inlineStr">
-        <is>
-          <t>D08 Flash 分区设计</t>
-        </is>
-      </c>
     </row>
     <row r="16" ht="33" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>2.6</t>
+          <t>2.7</t>
         </is>
       </c>
       <c r="B16" s="9" t="n"/>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>CAN 通信设计</t>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>设计内部评审</t>
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>46216</v>
+        <v>46218</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>46217</v>
+        <v>46218</v>
       </c>
       <c r="F16" s="4" t="inlineStr"/>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>嵌入式开发工程师</t>
-        </is>
-      </c>
-      <c r="H16" s="8" t="inlineStr">
-        <is>
-          <t>D09 CAN 通信设计</t>
+          <t>项目团队</t>
         </is>
       </c>
     </row>
     <row r="17" ht="33" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>2.7</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="n"/>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>设计内部评审</t>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>软件开发 — Bootloader</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>MCU 底层初始化及配置</t>
         </is>
       </c>
       <c r="D17" s="5" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>46218</v>
+        <v>46220</v>
       </c>
       <c r="F17" s="4" t="inlineStr"/>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>项目团队</t>
-        </is>
-      </c>
-      <c r="H17" s="8" t="inlineStr">
-        <is>
-          <t>设计评审记录</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="16.5" customHeight="1">
-      <c r="A18" s="3" t="inlineStr"/>
-      <c r="B18" s="3" t="inlineStr"/>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>阶段二 小计</t>
-        </is>
-      </c>
-      <c r="D18" s="11" t="n">
-        <v>46202</v>
-      </c>
-      <c r="E18" s="11" t="n">
-        <v>46218</v>
+          <t>嵌入式开发工程师</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="33" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="n"/>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>CAN 驱动开发</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>46223</v>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>46224</v>
       </c>
       <c r="F18" s="4" t="inlineStr"/>
-      <c r="G18" s="4" t="inlineStr"/>
-      <c r="H18" s="4" t="inlineStr"/>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>嵌入式开发工程师</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="33" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>3.1</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>软件开发 — Bootloader</t>
-        </is>
-      </c>
-      <c r="C19" s="8" t="inlineStr">
-        <is>
-          <t>MCU 底层初始化及配置</t>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="n"/>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>CAN-TP 传输层</t>
         </is>
       </c>
       <c r="D19" s="5" t="n">
-        <v>46219</v>
+        <v>46225</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>46220</v>
+        <v>46230</v>
       </c>
       <c r="F19" s="4" t="inlineStr"/>
       <c r="G19" s="4" t="inlineStr">
@@ -1115,29 +1041,24 @@
           <t>嵌入式开发工程师</t>
         </is>
       </c>
-      <c r="H19" s="8" t="inlineStr">
-        <is>
-          <t>凌鸥芯片适配</t>
-        </is>
-      </c>
     </row>
     <row r="20" ht="33" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>3.2</t>
-        </is>
-      </c>
-      <c r="B20" s="9" t="n"/>
-      <c r="C20" s="8" t="inlineStr">
-        <is>
-          <t>CAN 驱动开发</t>
+          <t>3.4</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="n"/>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>UDS 诊断栈</t>
         </is>
       </c>
       <c r="D20" s="5" t="n">
-        <v>46223</v>
+        <v>46231</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>46224</v>
+        <v>46238</v>
       </c>
       <c r="F20" s="4" t="inlineStr"/>
       <c r="G20" s="4" t="inlineStr">
@@ -1145,29 +1066,24 @@
           <t>嵌入式开发工程师</t>
         </is>
       </c>
-      <c r="H20" s="8" t="inlineStr">
-        <is>
-          <t>初始化/收发/滤波/中断</t>
-        </is>
-      </c>
     </row>
     <row r="21" ht="33" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>3.3</t>
-        </is>
-      </c>
-      <c r="B21" s="9" t="n"/>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>CAN-TP 传输层</t>
+          <t>3.5</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="n"/>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>安全信息访问</t>
         </is>
       </c>
       <c r="D21" s="5" t="n">
-        <v>46225</v>
+        <v>46239</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>46230</v>
+        <v>46244</v>
       </c>
       <c r="F21" s="4" t="inlineStr"/>
       <c r="G21" s="4" t="inlineStr">
@@ -1175,29 +1091,24 @@
           <t>嵌入式开发工程师</t>
         </is>
       </c>
-      <c r="H21" s="8" t="inlineStr">
-        <is>
-          <t>单帧/多帧/流控/定时</t>
-        </is>
-      </c>
     </row>
     <row r="22" ht="33" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>3.4</t>
-        </is>
-      </c>
-      <c r="B22" s="9" t="n"/>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>UDS 诊断栈</t>
+          <t>3.6</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="n"/>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Flash 擦写驱动 + CRC32</t>
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>46231</v>
+        <v>46245</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>46238</v>
+        <v>46246</v>
       </c>
       <c r="F22" s="4" t="inlineStr"/>
       <c r="G22" s="4" t="inlineStr">
@@ -1205,29 +1116,24 @@
           <t>嵌入式开发工程师</t>
         </is>
       </c>
-      <c r="H22" s="8" t="inlineStr">
-        <is>
-          <t>10个SID服务实现</t>
-        </is>
-      </c>
     </row>
     <row r="23" ht="33" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>3.5</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="n"/>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>安全信息访问</t>
+          <t>3.7</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="n"/>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>刷写状态机 + NRC + 跳步约束</t>
         </is>
       </c>
       <c r="D23" s="5" t="n">
-        <v>46239</v>
+        <v>46247</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>46244</v>
+        <v>46251</v>
       </c>
       <c r="F23" s="4" t="inlineStr"/>
       <c r="G23" s="4" t="inlineStr">
@@ -1235,29 +1141,24 @@
           <t>嵌入式开发工程师</t>
         </is>
       </c>
-      <c r="H23" s="8" t="inlineStr">
-        <is>
-          <t>含算法验证和测试向量比对</t>
-        </is>
-      </c>
     </row>
     <row r="24" ht="33" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>3.6</t>
+          <t>3.8</t>
         </is>
       </c>
       <c r="B24" s="9" t="n"/>
-      <c r="C24" s="8" t="inlineStr">
-        <is>
-          <t>Flash 擦写驱动 + CRC32</t>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Bootloader 集成调试</t>
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>46245</v>
+        <v>46252</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>46246</v>
+        <v>46255</v>
       </c>
       <c r="F24" s="4" t="inlineStr"/>
       <c r="G24" s="4" t="inlineStr">
@@ -1265,29 +1166,28 @@
           <t>嵌入式开发工程师</t>
         </is>
       </c>
-      <c r="H24" s="8" t="inlineStr">
-        <is>
-          <t>含硬件CRC模块调用</t>
-        </is>
-      </c>
     </row>
     <row r="25" ht="33" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>3.7</t>
-        </is>
-      </c>
-      <c r="B25" s="9" t="n"/>
-      <c r="C25" s="8" t="inlineStr">
-        <is>
-          <t>刷写状态机 + NRC + 跳步约束</t>
+          <t>3.9</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>软件开发 — Application</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>App 初始化 + CAN 驱动</t>
         </is>
       </c>
       <c r="D25" s="5" t="n">
-        <v>46247</v>
+        <v>46258</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>46251</v>
+        <v>46259</v>
       </c>
       <c r="F25" s="4" t="inlineStr"/>
       <c r="G25" s="4" t="inlineStr">
@@ -1295,29 +1195,24 @@
           <t>嵌入式开发工程师</t>
         </is>
       </c>
-      <c r="H25" s="8" t="inlineStr">
-        <is>
-          <t>16条跳步规则实现</t>
-        </is>
-      </c>
     </row>
     <row r="26" ht="33" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>3.8</t>
-        </is>
-      </c>
-      <c r="B26" s="10" t="n"/>
-      <c r="C26" s="8" t="inlineStr">
-        <is>
-          <t>Bootloader 集成调试</t>
+          <t>3.10</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="n"/>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>UDS 诊断栈</t>
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>46252</v>
+        <v>46260</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>46255</v>
+        <v>46265</v>
       </c>
       <c r="F26" s="4" t="inlineStr"/>
       <c r="G26" s="4" t="inlineStr">
@@ -1325,51 +1220,49 @@
           <t>嵌入式开发工程师</t>
         </is>
       </c>
-      <c r="H26" s="8" t="inlineStr">
-        <is>
-          <t>端到端刷写流程联调</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="16.5" customHeight="1">
-      <c r="A27" s="3" t="inlineStr"/>
-      <c r="B27" s="3" t="inlineStr"/>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>BT 开发 小计</t>
-        </is>
-      </c>
-      <c r="D27" s="11" t="n">
-        <v>46219</v>
-      </c>
-      <c r="E27" s="11" t="n">
-        <v>46255</v>
+    </row>
+    <row r="27" ht="33" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>3.11</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="n"/>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>DID 管理模块</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>46266</v>
+      </c>
+      <c r="E27" s="5" t="n">
+        <v>46267</v>
       </c>
       <c r="F27" s="4" t="inlineStr"/>
-      <c r="G27" s="4" t="inlineStr"/>
-      <c r="H27" s="4" t="inlineStr"/>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>嵌入式开发工程师</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="33" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>3.9</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>软件开发 — Application</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>App 初始化 + CAN 驱动</t>
+          <t>3.12</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="n"/>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>DTC 管理模块</t>
         </is>
       </c>
       <c r="D28" s="5" t="n">
-        <v>46258</v>
+        <v>46268</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>46259</v>
+        <v>46269</v>
       </c>
       <c r="F28" s="4" t="inlineStr"/>
       <c r="G28" s="4" t="inlineStr">
@@ -1377,29 +1270,24 @@
           <t>嵌入式开发工程师</t>
         </is>
       </c>
-      <c r="H28" s="8" t="inlineStr">
-        <is>
-          <t>部分代码共用</t>
-        </is>
-      </c>
     </row>
     <row r="29" ht="33" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>3.10</t>
-        </is>
-      </c>
-      <c r="B29" s="9" t="n"/>
-      <c r="C29" s="8" t="inlineStr">
-        <is>
-          <t>UDS 诊断栈</t>
+          <t>3.13</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="n"/>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>编程前条件检查</t>
         </is>
       </c>
       <c r="D29" s="5" t="n">
-        <v>46260</v>
+        <v>46272</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>46265</v>
+        <v>46273</v>
       </c>
       <c r="F29" s="4" t="inlineStr"/>
       <c r="G29" s="4" t="inlineStr">
@@ -1407,29 +1295,24 @@
           <t>嵌入式开发工程师</t>
         </is>
       </c>
-      <c r="H29" s="8" t="inlineStr">
-        <is>
-          <t>完整诊断服务</t>
-        </is>
-      </c>
     </row>
     <row r="30" ht="33" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>3.11</t>
-        </is>
-      </c>
-      <c r="B30" s="9" t="n"/>
-      <c r="C30" s="8" t="inlineStr">
-        <is>
-          <t>DID 管理模块</t>
+          <t>3.14</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="n"/>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>风扇控制功能集成</t>
         </is>
       </c>
       <c r="D30" s="5" t="n">
-        <v>46266</v>
+        <v>46274</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>46267</v>
+        <v>46280</v>
       </c>
       <c r="F30" s="4" t="inlineStr"/>
       <c r="G30" s="4" t="inlineStr">
@@ -1437,29 +1320,24 @@
           <t>嵌入式开发工程师</t>
         </is>
       </c>
-      <c r="H30" s="8" t="inlineStr">
-        <is>
-          <t>10+ 个 DID 读写</t>
-        </is>
-      </c>
     </row>
     <row r="31" ht="33" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>3.12</t>
+          <t>3.15</t>
         </is>
       </c>
       <c r="B31" s="9" t="n"/>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>DTC 管理模块</t>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Application 集成调试</t>
         </is>
       </c>
       <c r="D31" s="5" t="n">
-        <v>46268</v>
+        <v>46281</v>
       </c>
       <c r="E31" s="5" t="n">
-        <v>46269</v>
+        <v>46283</v>
       </c>
       <c r="F31" s="4" t="inlineStr"/>
       <c r="G31" s="4" t="inlineStr">
@@ -1467,249 +1345,236 @@
           <t>嵌入式开发工程师</t>
         </is>
       </c>
-      <c r="H31" s="8" t="inlineStr">
-        <is>
-          <t>0x14/0x19 服务</t>
-        </is>
-      </c>
     </row>
     <row r="32" ht="33" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>3.13</t>
-        </is>
-      </c>
-      <c r="B32" s="9" t="n"/>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>编程前条件检查</t>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>测试验证</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>单元测试（关键模块）</t>
         </is>
       </c>
       <c r="D32" s="5" t="n">
-        <v>46272</v>
+        <v>46286</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>46273</v>
+        <v>46287</v>
       </c>
       <c r="F32" s="4" t="inlineStr"/>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>嵌入式开发工程师</t>
-        </is>
-      </c>
-      <c r="H32" s="8" t="inlineStr">
-        <is>
-          <t>CAN 信号接收+条件判断</t>
+          <t>开发+测试</t>
         </is>
       </c>
     </row>
     <row r="33" ht="33" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>3.14</t>
-        </is>
-      </c>
-      <c r="B33" s="9" t="n"/>
-      <c r="C33" s="8" t="inlineStr">
-        <is>
-          <t>风扇控制功能集成</t>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="n"/>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Bootloader 刷写流程测试</t>
         </is>
       </c>
       <c r="D33" s="5" t="n">
-        <v>46274</v>
+        <v>46288</v>
       </c>
       <c r="E33" s="5" t="n">
-        <v>46280</v>
+        <v>46289</v>
       </c>
       <c r="F33" s="4" t="inlineStr"/>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>嵌入式开发工程师</t>
-        </is>
-      </c>
-      <c r="H33" s="8" t="inlineStr">
-        <is>
-          <t>PWM+ADC</t>
+          <t>测试工程师</t>
         </is>
       </c>
     </row>
     <row r="34" ht="33" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>3.15</t>
-        </is>
-      </c>
-      <c r="B34" s="10" t="n"/>
-      <c r="C34" s="8" t="inlineStr">
-        <is>
-          <t>Application 集成调试</t>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="n"/>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>诊断功能测试</t>
         </is>
       </c>
       <c r="D34" s="5" t="n">
-        <v>46281</v>
+        <v>46293</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>46283</v>
+        <v>46295</v>
       </c>
       <c r="F34" s="4" t="inlineStr"/>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>嵌入式开发工程师</t>
-        </is>
-      </c>
-      <c r="H34" s="8" t="inlineStr">
-        <is>
-          <t>端到端诊断功能联调</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="16.5" customHeight="1">
-      <c r="A35" s="3" t="inlineStr"/>
-      <c r="B35" s="3" t="inlineStr"/>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>App 开发 小计</t>
-        </is>
-      </c>
-      <c r="D35" s="11" t="n">
-        <v>46258</v>
-      </c>
-      <c r="E35" s="11" t="n">
-        <v>46283</v>
+          <t>测试工程师</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="33" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="n"/>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>安全访问测试</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E35" s="5" t="n">
+        <v>46304</v>
       </c>
       <c r="F35" s="4" t="inlineStr"/>
-      <c r="G35" s="4" t="inlineStr"/>
-      <c r="H35" s="4" t="inlineStr"/>
-    </row>
-    <row r="36" ht="16.5" customHeight="1">
-      <c r="A36" s="3" t="inlineStr"/>
-      <c r="B36" s="3" t="inlineStr"/>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>阶段三 合计</t>
-        </is>
-      </c>
-      <c r="D36" s="11" t="n">
-        <v>46219</v>
-      </c>
-      <c r="E36" s="11" t="n">
-        <v>46283</v>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>测试工程师</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="33" customHeight="1">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="B36" s="8" t="n"/>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>BT↔App 集成测试</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E36" s="5" t="n">
+        <v>46309</v>
       </c>
       <c r="F36" s="4" t="inlineStr"/>
-      <c r="G36" s="4" t="inlineStr"/>
-      <c r="H36" s="4" t="inlineStr"/>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>测试工程师</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="33" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>4.1</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>测试验证</t>
-        </is>
-      </c>
-      <c r="C37" s="8" t="inlineStr">
-        <is>
-          <t>单元测试（关键模块）</t>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="B37" s="8" t="n"/>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Bug 修复与回归测试</t>
         </is>
       </c>
       <c r="D37" s="5" t="n">
-        <v>46286</v>
+        <v>46310</v>
       </c>
       <c r="E37" s="5" t="n">
-        <v>46287</v>
+        <v>46315</v>
       </c>
       <c r="F37" s="4" t="inlineStr"/>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>开发+测试</t>
-        </is>
-      </c>
-      <c r="H37" s="8" t="inlineStr">
-        <is>
-          <t>AES/CRC/Flash/CAN-TP</t>
+          <t>开发工程师</t>
         </is>
       </c>
     </row>
     <row r="38" ht="33" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="B38" s="9" t="n"/>
-      <c r="C38" s="8" t="inlineStr">
-        <is>
-          <t>Bootloader 刷写流程测试</t>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>台架联调关门</t>
         </is>
       </c>
       <c r="D38" s="5" t="n">
-        <v>46288</v>
+        <v>46316</v>
       </c>
       <c r="E38" s="5" t="n">
-        <v>46289</v>
-      </c>
-      <c r="F38" s="4" t="inlineStr"/>
+        <v>46317</v>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>台架通过</t>
+        </is>
+      </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
           <t>测试工程师</t>
-        </is>
-      </c>
-      <c r="H38" s="8" t="inlineStr">
-        <is>
-          <t>正常+16条异常路径</t>
         </is>
       </c>
     </row>
     <row r="39" ht="33" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>4.3</t>
-        </is>
-      </c>
-      <c r="B39" s="9" t="n"/>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>诊断功能测试</t>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>信息安全文档</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>信息安全技术规范填充</t>
         </is>
       </c>
       <c r="D39" s="5" t="n">
-        <v>46293</v>
+        <v>46219</v>
       </c>
       <c r="E39" s="5" t="n">
-        <v>46295</v>
+        <v>46220</v>
       </c>
       <c r="F39" s="4" t="inlineStr"/>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>测试工程师</t>
-        </is>
-      </c>
-      <c r="H39" s="8" t="inlineStr">
-        <is>
-          <t>全SID/全会话/全NRC</t>
+          <t>系统工程师</t>
         </is>
       </c>
     </row>
     <row r="40" ht="33" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>4.4</t>
-        </is>
-      </c>
-      <c r="B40" s="9" t="n"/>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>安全访问测试</t>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="B40" s="8" t="n"/>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>信息安全测试用例编写</t>
         </is>
       </c>
       <c r="D40" s="5" t="n">
-        <v>46303</v>
+        <v>46223</v>
       </c>
       <c r="E40" s="5" t="n">
-        <v>46304</v>
+        <v>46224</v>
       </c>
       <c r="F40" s="4" t="inlineStr"/>
       <c r="G40" s="4" t="inlineStr">
@@ -1717,446 +1582,181 @@
           <t>测试工程师</t>
         </is>
       </c>
-      <c r="H40" s="8" t="inlineStr">
-        <is>
-          <t>算法正确性+锁定机制</t>
-        </is>
-      </c>
     </row>
     <row r="41" ht="33" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>4.5</t>
-        </is>
-      </c>
-      <c r="B41" s="9" t="n"/>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>BT↔App 集成测试</t>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="n"/>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>CIA 接口协议确认与修订</t>
         </is>
       </c>
       <c r="D41" s="5" t="n">
-        <v>46307</v>
+        <v>46225</v>
       </c>
       <c r="E41" s="5" t="n">
-        <v>46309</v>
+        <v>46226</v>
       </c>
       <c r="F41" s="4" t="inlineStr"/>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>测试工程师</t>
-        </is>
-      </c>
-      <c r="H41" s="8" t="inlineStr">
-        <is>
-          <t>刷写闭环+会话切换</t>
+          <t>项目经理</t>
         </is>
       </c>
     </row>
     <row r="42" ht="33" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>5.4</t>
         </is>
       </c>
       <c r="B42" s="9" t="n"/>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>Bug 修复与回归测试</t>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>信息安全评审</t>
         </is>
       </c>
       <c r="D42" s="5" t="n">
-        <v>46310</v>
+        <v>46227</v>
       </c>
       <c r="E42" s="5" t="n">
-        <v>46315</v>
+        <v>46227</v>
       </c>
       <c r="F42" s="4" t="inlineStr"/>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>开发工程师</t>
-        </is>
-      </c>
-      <c r="H42" s="8" t="inlineStr">
-        <is>
-          <t>问题修复验证</t>
+          <t>项目团队</t>
         </is>
       </c>
     </row>
     <row r="43" ht="33" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>4.7</t>
-        </is>
-      </c>
-      <c r="B43" s="10" t="n"/>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>台架联调关门</t>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>交付与客户支持</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>交样软件冻结</t>
         </is>
       </c>
       <c r="D43" s="5" t="n">
-        <v>46316</v>
+        <v>46318</v>
       </c>
       <c r="E43" s="5" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>台架通过</t>
+          <t>交样</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>测试工程师</t>
-        </is>
-      </c>
-      <c r="H43" s="8" t="inlineStr">
-        <is>
-          <t>台架联调记录</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="16.5" customHeight="1">
-      <c r="A44" s="3" t="inlineStr"/>
-      <c r="B44" s="3" t="inlineStr"/>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>阶段四 小计</t>
-        </is>
-      </c>
-      <c r="D44" s="11" t="n">
-        <v>46286</v>
-      </c>
-      <c r="E44" s="11" t="n">
-        <v>46317</v>
+          <t>开发工程师</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="33" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="B44" s="8" t="n"/>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>版本发布说明编写</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="n">
+        <v>46321</v>
+      </c>
+      <c r="E44" s="5" t="n">
+        <v>46321</v>
       </c>
       <c r="F44" s="4" t="inlineStr"/>
-      <c r="G44" s="4" t="inlineStr"/>
-      <c r="H44" s="4" t="inlineStr"/>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>开发工程师</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="33" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>5.1</t>
-        </is>
-      </c>
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>信息安全文档</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>信息安全技术规范填充</t>
+          <t>6.3</t>
+        </is>
+      </c>
+      <c r="B45" s="8" t="n"/>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>交付评审</t>
         </is>
       </c>
       <c r="D45" s="5" t="n">
-        <v>46219</v>
+        <v>46322</v>
       </c>
       <c r="E45" s="5" t="n">
-        <v>46220</v>
+        <v>46322</v>
       </c>
       <c r="F45" s="4" t="inlineStr"/>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>系统工程师</t>
-        </is>
-      </c>
-      <c r="H45" s="8" t="inlineStr">
-        <is>
-          <t>D10 CS100120-027C</t>
+          <t>项目团队+客户</t>
         </is>
       </c>
     </row>
     <row r="46" ht="33" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>5.2</t>
+          <t>6.4</t>
         </is>
       </c>
       <c r="B46" s="9" t="n"/>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>信息安全测试用例编写</t>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>客户侧验证技术支持</t>
         </is>
       </c>
       <c r="D46" s="5" t="n">
-        <v>46223</v>
+        <v>46323</v>
       </c>
       <c r="E46" s="5" t="n">
-        <v>46224</v>
-      </c>
-      <c r="F46" s="4" t="inlineStr"/>
+        <v>46325</v>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>开发关闭</t>
+        </is>
+      </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
-          <t>测试工程师</t>
-        </is>
-      </c>
-      <c r="H46" s="8" t="inlineStr">
-        <is>
-          <t>D11 CS100120-030C</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="33" customHeight="1">
-      <c r="A47" s="4" t="inlineStr">
-        <is>
-          <t>5.3</t>
-        </is>
-      </c>
-      <c r="B47" s="9" t="n"/>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>CIA 接口协议确认与修订</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="n">
-        <v>46225</v>
-      </c>
-      <c r="E47" s="5" t="n">
-        <v>46226</v>
-      </c>
-      <c r="F47" s="4" t="inlineStr"/>
-      <c r="G47" s="4" t="inlineStr">
-        <is>
-          <t>项目经理</t>
-        </is>
-      </c>
-      <c r="H47" s="8" t="inlineStr">
-        <is>
-          <t>D12 CS100120-045C</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="33" customHeight="1">
-      <c r="A48" s="4" t="inlineStr">
-        <is>
-          <t>5.4</t>
-        </is>
-      </c>
-      <c r="B48" s="10" t="n"/>
-      <c r="C48" s="8" t="inlineStr">
-        <is>
-          <t>信息安全评审</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="n">
-        <v>46227</v>
-      </c>
-      <c r="E48" s="5" t="n">
-        <v>46227</v>
-      </c>
-      <c r="F48" s="4" t="inlineStr"/>
-      <c r="G48" s="4" t="inlineStr">
-        <is>
-          <t>项目团队</t>
-        </is>
-      </c>
-      <c r="H48" s="8" t="inlineStr">
-        <is>
-          <t>评审记录</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="16.5" customHeight="1">
-      <c r="A49" s="3" t="inlineStr"/>
-      <c r="B49" s="3" t="inlineStr"/>
-      <c r="C49" s="3" t="inlineStr">
-        <is>
-          <t>阶段五 小计</t>
-        </is>
-      </c>
-      <c r="D49" s="11" t="n">
-        <v>46219</v>
-      </c>
-      <c r="E49" s="11" t="n">
-        <v>46227</v>
-      </c>
-      <c r="F49" s="4" t="inlineStr"/>
-      <c r="G49" s="4" t="inlineStr"/>
-      <c r="H49" s="4" t="inlineStr"/>
-    </row>
-    <row r="50" ht="33" customHeight="1">
-      <c r="A50" s="4" t="inlineStr">
-        <is>
-          <t>6.1</t>
-        </is>
-      </c>
-      <c r="B50" s="4" t="inlineStr">
-        <is>
-          <t>交付与客户支持</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="inlineStr">
-        <is>
-          <t>交样软件冻结</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="n">
-        <v>46318</v>
-      </c>
-      <c r="E50" s="5" t="n">
-        <v>46318</v>
-      </c>
-      <c r="F50" s="4" t="inlineStr">
-        <is>
-          <t>交样</t>
-        </is>
-      </c>
-      <c r="G50" s="4" t="inlineStr">
-        <is>
           <t>开发工程师</t>
         </is>
       </c>
-      <c r="H50" s="8" t="inlineStr">
-        <is>
-          <t>冻结版本号及校验和</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="33" customHeight="1">
-      <c r="A51" s="4" t="inlineStr">
-        <is>
-          <t>6.2</t>
-        </is>
-      </c>
-      <c r="B51" s="9" t="n"/>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>版本发布说明编写</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="n">
-        <v>46321</v>
-      </c>
-      <c r="E51" s="5" t="n">
-        <v>46321</v>
-      </c>
-      <c r="F51" s="4" t="inlineStr"/>
-      <c r="G51" s="4" t="inlineStr">
-        <is>
-          <t>开发工程师</t>
-        </is>
-      </c>
-      <c r="H51" s="8" t="inlineStr">
-        <is>
-          <t>D17 版本发布说明</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="33" customHeight="1">
-      <c r="A52" s="4" t="inlineStr">
-        <is>
-          <t>6.3</t>
-        </is>
-      </c>
-      <c r="B52" s="9" t="n"/>
-      <c r="C52" s="8" t="inlineStr">
-        <is>
-          <t>交付评审</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="n">
-        <v>46322</v>
-      </c>
-      <c r="E52" s="5" t="n">
-        <v>46322</v>
-      </c>
-      <c r="F52" s="4" t="inlineStr"/>
-      <c r="G52" s="4" t="inlineStr">
-        <is>
-          <t>项目团队+客户</t>
-        </is>
-      </c>
-      <c r="H52" s="8" t="inlineStr">
-        <is>
-          <t>评审记录</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="33" customHeight="1">
-      <c r="A53" s="4" t="inlineStr">
-        <is>
-          <t>6.4</t>
-        </is>
-      </c>
-      <c r="B53" s="10" t="n"/>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>客户侧验证技术支持</t>
-        </is>
-      </c>
-      <c r="D53" s="5" t="n">
-        <v>46323</v>
-      </c>
-      <c r="E53" s="5" t="n">
-        <v>46325</v>
-      </c>
-      <c r="F53" s="4" t="inlineStr">
-        <is>
-          <t>开发关闭</t>
-        </is>
-      </c>
-      <c r="G53" s="4" t="inlineStr">
-        <is>
-          <t>开发工程师</t>
-        </is>
-      </c>
-      <c r="H53" s="8" t="inlineStr">
-        <is>
-          <t>现场/远程支持</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="16.5" customHeight="1">
-      <c r="A54" s="3" t="inlineStr"/>
-      <c r="B54" s="3" t="inlineStr"/>
-      <c r="C54" s="3" t="inlineStr">
-        <is>
-          <t>阶段六 小计</t>
-        </is>
-      </c>
-      <c r="D54" s="11" t="n">
-        <v>46318</v>
-      </c>
-      <c r="E54" s="11" t="n">
-        <v>46325</v>
-      </c>
-      <c r="F54" s="4" t="inlineStr"/>
-      <c r="G54" s="4" t="inlineStr"/>
-      <c r="H54" s="4" t="inlineStr"/>
-    </row>
-    <row r="55" ht="16.5" customHeight="1">
-      <c r="A55" s="3" t="inlineStr"/>
-      <c r="B55" s="3" t="inlineStr"/>
-      <c r="C55" s="3" t="inlineStr">
-        <is>
-          <t>项目合计</t>
-        </is>
-      </c>
-      <c r="D55" s="11" t="n">
-        <v>46188</v>
-      </c>
-      <c r="E55" s="11" t="n">
-        <v>46325</v>
-      </c>
-      <c r="F55" s="4" t="inlineStr"/>
-      <c r="G55" s="4" t="inlineStr"/>
-      <c r="H55" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H4"/>
+  <autoFilter ref="A4:G4"/>
   <mergeCells count="9">
-    <mergeCell ref="B28:B34"/>
-    <mergeCell ref="B50:B53"/>
-    <mergeCell ref="B19:B26"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="B45:B48"/>
-    <mergeCell ref="F3:H3"/>
-    <mergeCell ref="B37:B43"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="B17:B24"/>
+    <mergeCell ref="B32:B38"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="B10:B16"/>
+    <mergeCell ref="B43:B46"/>
+    <mergeCell ref="B39:B42"/>
+    <mergeCell ref="B25:B31"/>
     <mergeCell ref="B5:B9"/>
-    <mergeCell ref="B11:B17"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="1" fitToWidth="1"/>

</xml_diff>